<commit_message>
feat: implement robust fuzzy-matching PDF reporting engine with embedded charts
</commit_message>
<xml_diff>
--- a/exported_report.xlsx
+++ b/exported_report.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,10 +43,6 @@
     <font>
       <b val="1"/>
       <sz val="14"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00555555"/>
     </font>
   </fonts>
   <fills count="3">
@@ -75,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -84,7 +80,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -159,136 +154,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>1</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="15240000" cy="9525000"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>32</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="15240000" cy="9525000"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Image 2" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>63</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="15240000" cy="9525000"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="3" name="Image 3" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>94</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="15240000" cy="9525000"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="4" name="Image 4" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId4"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>125</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="15240000" cy="9525000"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="5" name="Image 5" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId5"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -691,7 +556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -707,7 +572,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Analysis of 5 records across 3 columns reveals 1 critical findings. The top 3 Product values (Y, Z, X) account for 100.0% of total Sales.</t>
+          <t>Strategic Brief: The E-commerce system is operating at a scale of 5 records with stable high-level consistency. Analytical focus is centered on the optimization of key metrics across all categorical segments. No secondary drivers met the strategic significance threshold at this time. Current risk assessment identifies 1 critical structural anomalies requiring immediate executive intervention. Strategic implication: Future performance gains will require a targeted focus on key metrics optimization.</t>
         </is>
       </c>
     </row>
@@ -721,7 +586,10 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>• Top 3 Product by Sales: The top 3 Product values (Y, Z, X) account for 100.0% of total Sales.</t>
+          <t>• No Significant Insights Detected: **STRATEGIC OBSERVATION**: The current analytical session did not exhibit patterns meeting the high-impact strategic threshold.
+**WHY IT MATTERS**: Data homogeneity or limited variability may be preventing the isolation of distinct business drivers.
+**SUPPORTING EVIDENCE**: Statistical variance within acceptable margins.
+**DECISION IMPLICATION**: Collect more granular data or refine the analytical focus variables to isolate deeper trends.</t>
         </is>
       </c>
     </row>
@@ -729,13 +597,6 @@
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Recommendations</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>• Focus resources on top-performing Product categories to maximize Sales.</t>
         </is>
       </c>
     </row>
@@ -750,7 +611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A155"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -759,90 +620,60 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Sales by Sales</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <t>Insight: 5 categories (ideal) • Balanced distribution • Shows distribution shape + outliers</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
-        <is>
-          <t>Sales Summary</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="6" t="inlineStr">
-        <is>
-          <t>Insight: Statistical summary with confidence notches</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="5" t="inlineStr">
-        <is>
-          <t>Product Breakdown</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Insight: </t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr"/>
-    </row>
-    <row r="94">
-      <c r="A94" s="5" t="inlineStr">
+          <t>Which Product performs best in each Region?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>[Image could not be generated: You must install Pillow to fetch image objects]</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Which Product has the most orders?</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>[Image could not be generated: You must install Pillow to fetch image objects]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Sales Distribution</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>[Image could not be generated: You must install Pillow to fetch image objects]</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Sales by Product</t>
         </is>
       </c>
     </row>
-    <row r="121">
-      <c r="A121" s="6" t="inlineStr">
-        <is>
-          <t>Insight: 3 categories (ideal) • Balanced distribution</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="inlineStr"/>
-    </row>
-    <row r="125">
-      <c r="A125" s="5" t="inlineStr">
-        <is>
-          <t>Product by Sales</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Insight: </t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="inlineStr"/>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>[Image could not be generated: You must install Pillow to fetch image objects]</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>